<commit_message>
Add project CRUD API and tests
</commit_message>
<xml_diff>
--- a/05_FASTAPI/doc/FastAPI_India_Market_Research_API.xlsx
+++ b/05_FASTAPI/doc/FastAPI_India_Market_Research_API.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\learning_products\05_FASTAPI\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E90AAA-5972-461C-A755-24648CCFA3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0ED6D76-6EE7-4261-BBA4-A82AF40A1283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{525C93EA-9DB4-478D-A5E6-B36F2A5163DF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{525C93EA-9DB4-478D-A5E6-B36F2A5163DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Schematic diagram" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="test_result①" sheetId="6" r:id="rId7"/>
     <sheet name="test_result②" sheetId="7" r:id="rId8"/>
     <sheet name="test_result③" sheetId="8" r:id="rId9"/>
-    <sheet name="Sheet2" sheetId="10" r:id="rId10"/>
+    <sheet name="test_result④" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="134">
   <si>
     <t>app/</t>
   </si>
@@ -285,10 +285,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>└──company.py</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>├──user.cpython-313.pyc</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -440,10 +436,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>└──test_companies.py</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>├──env.docker</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -461,6 +453,86 @@
   </si>
   <si>
     <t>├── Dockerfile</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>├─projects.py</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>├──projects.py</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>└──projects.py</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>└──test_projects.py</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>├──test_companies.py</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/projects/</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/projects/{project_id}</t>
+  </si>
+  <si>
+    <t>Read projects</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/projects/{project_id}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/projects/company/{company_id}</t>
+  </si>
+  <si>
+    <t>/projects</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>company_id</t>
+  </si>
+  <si>
+    <t>project_name</t>
+  </si>
+  <si>
+    <t>project_type</t>
+  </si>
+  <si>
+    <t>budget</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>start_date</t>
+  </si>
+  <si>
+    <t>end_date</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>projects</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Pytest</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -468,7 +540,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,6 +577,12 @@
       <name val="Meiryo UI"/>
       <family val="3"/>
       <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -657,7 +735,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -723,6 +801,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1509,6 +1593,55 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>328262</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>137577</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="図 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2F022891-7211-D1AC-27EB-3BC3E0ACD1DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="91440" y="586740"/>
+          <a:ext cx="6942422" cy="4808637"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
   <a:themeElements>
@@ -1807,7 +1940,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59C5FE2C-F88C-40CF-B11A-6EB7AEAAC90D}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1817,30 +1950,37 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AA7A343-3B7E-438B-8077-FC6305E3DEFF}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <dimension ref="A2"/>
+  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetData>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8876FB0B-A80E-4DB2-9C25-5AA7068C16FC}">
-  <dimension ref="A2:C61"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <dimension ref="A2:C66"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <sheetData>
-    <row r="2" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A4" t="s">
         <v>50</v>
       </c>
@@ -1848,7 +1988,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1856,12 +1996,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -1869,7 +2009,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -1880,7 +2020,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -1891,7 +2031,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A10" t="s">
         <v>50</v>
       </c>
@@ -1902,7 +2042,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A11" t="s">
         <v>50</v>
       </c>
@@ -1910,7 +2050,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -1918,384 +2058,433 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" ht="17.399999999999999" customHeight="1">
       <c r="A13" t="s">
         <v>50</v>
       </c>
       <c r="B13" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="16" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B16" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" t="s">
+    <row r="17" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" t="s">
+    <row r="18" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" t="s">
+    <row r="19" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" t="s">
+    <row r="20" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" t="s">
+    <row r="21" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>50</v>
-      </c>
-      <c r="B22" t="s">
+    <row r="24" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>50</v>
-      </c>
-      <c r="B23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" t="s">
+    <row r="25" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" t="s">
+    <row r="26" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" t="s">
+    <row r="27" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A27" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" t="s">
+    <row r="28" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" t="s">
+    <row r="29" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" t="s">
+    <row r="30" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A31" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A33" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A34" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" t="s">
+        <v>50</v>
+      </c>
+      <c r="C34" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A35" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" t="s">
+        <v>50</v>
+      </c>
+      <c r="C35" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A36" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C36" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
-        <v>50</v>
-      </c>
-      <c r="B30" t="s">
+    <row r="37" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A37" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A39" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A40" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A41" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A42" t="s">
+        <v>50</v>
+      </c>
+      <c r="B42" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A44" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
-        <v>50</v>
-      </c>
-      <c r="B31" t="s">
-        <v>50</v>
-      </c>
-      <c r="C31" t="s">
+    <row r="45" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A45" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" t="s">
-        <v>50</v>
-      </c>
-      <c r="C32" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
-        <v>50</v>
-      </c>
-      <c r="B33" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" t="s">
+    <row r="46" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A46" t="s">
+        <v>50</v>
+      </c>
+      <c r="C46" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A47" t="s">
+        <v>50</v>
+      </c>
+      <c r="C47" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A48" t="s">
+        <v>50</v>
+      </c>
+      <c r="C48" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A49" t="s">
+        <v>50</v>
+      </c>
+      <c r="B49" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A50" t="s">
+        <v>50</v>
+      </c>
+      <c r="B50" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A51" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A52" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A53" t="s">
+        <v>50</v>
+      </c>
+      <c r="B53" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A55" t="s">
+        <v>50</v>
+      </c>
+      <c r="B55" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A56" t="s">
+        <v>50</v>
+      </c>
+      <c r="C56" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
-        <v>50</v>
-      </c>
-      <c r="B34" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>50</v>
-      </c>
-      <c r="B35" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
-        <v>50</v>
-      </c>
-      <c r="B36" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
-        <v>50</v>
-      </c>
-      <c r="B37" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
-        <v>50</v>
-      </c>
-      <c r="B38" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
-        <v>50</v>
-      </c>
-      <c r="B40" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
-        <v>50</v>
-      </c>
-      <c r="C41" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
-        <v>50</v>
-      </c>
-      <c r="C42" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
-        <v>50</v>
-      </c>
-      <c r="C43" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
-        <v>50</v>
-      </c>
-      <c r="C44" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A45" t="s">
-        <v>50</v>
-      </c>
-      <c r="B45" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A46" t="s">
-        <v>50</v>
-      </c>
-      <c r="B46" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
-        <v>50</v>
-      </c>
-      <c r="B47" t="s">
+    <row r="57" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A57" t="s">
+        <v>50</v>
+      </c>
+      <c r="C57" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A58" t="s">
+        <v>50</v>
+      </c>
+      <c r="B58" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
-        <v>50</v>
-      </c>
-      <c r="B48" t="s">
+    <row r="59" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A59" t="s">
+        <v>50</v>
+      </c>
+      <c r="B59" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="17.399999999999999" customHeight="1">
+      <c r="A60" t="s">
+        <v>50</v>
+      </c>
+      <c r="B60" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
         <v>107</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A49" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
-        <v>50</v>
-      </c>
-      <c r="B50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
-        <v>50</v>
-      </c>
-      <c r="C51" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
-        <v>50</v>
-      </c>
-      <c r="C52" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
-        <v>50</v>
-      </c>
-      <c r="B53" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
-        <v>50</v>
-      </c>
-      <c r="B54" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
-        <v>50</v>
-      </c>
-      <c r="B55" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A56" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A57" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A58" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A59" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A60" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A61" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2307,7 +2496,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55D3E2AD-F4D4-4A4C-BC53-A36DE7A07EB7}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2317,16 +2506,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A80FD98D-478F-42B4-AA74-6395C6F8B587}">
-  <dimension ref="B2:E15"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <dimension ref="B2:E23"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="2" max="2" width="12.3984375" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.19921875" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.09765625" style="19" customWidth="1"/>
+    <col min="4" max="4" width="33.3984375" style="19" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.69921875" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:5">
       <c r="B2" s="13" t="s">
         <v>32</v>
       </c>
@@ -2340,7 +2529,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:5">
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
@@ -2348,7 +2537,7 @@
       <c r="D3" s="7"/>
       <c r="E3" s="8"/>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:5">
       <c r="B4" s="2"/>
       <c r="C4" s="9" t="s">
         <v>8</v>
@@ -2360,7 +2549,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:5">
       <c r="B5" s="2"/>
       <c r="C5" s="9" t="s">
         <v>8</v>
@@ -2372,7 +2561,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:5">
       <c r="B6" s="6"/>
       <c r="C6" s="9" t="s">
         <v>9</v>
@@ -2384,7 +2573,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:5">
       <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
@@ -2392,7 +2581,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="4"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:5">
       <c r="B8" s="2"/>
       <c r="C8" s="9" t="s">
         <v>9</v>
@@ -2404,7 +2593,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:5">
       <c r="B9" s="2"/>
       <c r="C9" s="9" t="s">
         <v>8</v>
@@ -2416,7 +2605,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:5">
       <c r="B10" s="2"/>
       <c r="C10" s="9" t="s">
         <v>9</v>
@@ -2428,7 +2617,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:5">
       <c r="B11" s="2"/>
       <c r="C11" s="9" t="s">
         <v>10</v>
@@ -2440,7 +2629,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:5">
       <c r="B12" s="2"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
@@ -2452,7 +2641,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:5">
       <c r="B13" s="6"/>
       <c r="C13" s="9" t="s">
         <v>9</v>
@@ -2464,23 +2653,115 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:5">
       <c r="B14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="12"/>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B15" s="6"/>
+        <v>19</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="2:5">
+      <c r="B15" s="2"/>
       <c r="C15" s="9" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5">
+      <c r="B16" s="2"/>
+      <c r="C16" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="2"/>
+      <c r="C17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="2"/>
+      <c r="C18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5">
+      <c r="B19" s="2"/>
+      <c r="C19" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="2"/>
+      <c r="C20" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="18"/>
+      <c r="C21" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="12"/>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" s="6"/>
+      <c r="C23" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E23" s="10" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2492,14 +2773,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{992930C7-74C8-4FFB-9769-80CA943DB8EA}">
-  <dimension ref="B2:C16"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <dimension ref="B2:C36"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="2" max="2" width="10.796875" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.59765625" style="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:3">
       <c r="B2" s="15" t="s">
         <v>33</v>
       </c>
@@ -2507,67 +2788,67 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:3">
       <c r="B3" s="17"/>
       <c r="C3" s="16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:3">
       <c r="B4" s="17"/>
       <c r="C4" s="16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:3">
       <c r="B5" s="17"/>
       <c r="C5" s="16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:3">
       <c r="B6" s="17"/>
       <c r="C6" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:3">
       <c r="B7" s="17"/>
       <c r="C7" s="16" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:3">
       <c r="B8" s="17"/>
       <c r="C8" s="16" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:3">
       <c r="B9" s="17"/>
       <c r="C9" s="16" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:3">
       <c r="B10" s="17"/>
       <c r="C10" s="16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:3">
       <c r="B11" s="17"/>
       <c r="C11" s="16" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:3">
       <c r="B12" s="18"/>
       <c r="C12" s="16" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:3">
       <c r="B13" s="15" t="s">
         <v>44</v>
       </c>
@@ -2575,23 +2856,115 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:3">
       <c r="B14" s="17"/>
       <c r="C14" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:3">
       <c r="B15" s="17"/>
       <c r="C15" s="16" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:3">
       <c r="B16" s="18"/>
       <c r="C16" s="16" t="s">
         <v>47</v>
       </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="17"/>
+      <c r="C18" s="23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="17"/>
+      <c r="C19" s="23" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="17"/>
+      <c r="C20" s="23" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" s="17"/>
+      <c r="C21" s="23" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="17"/>
+      <c r="C22" s="23" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3">
+      <c r="B23" s="17"/>
+      <c r="C23" s="23" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3">
+      <c r="B24" s="17"/>
+      <c r="C24" s="23" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3">
+      <c r="B25" s="17"/>
+      <c r="C25" s="23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3">
+      <c r="B26" s="18"/>
+      <c r="C26" s="23" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3">
+      <c r="B27"/>
+    </row>
+    <row r="28" spans="2:3">
+      <c r="B28"/>
+    </row>
+    <row r="29" spans="2:3">
+      <c r="B29" s="22"/>
+    </row>
+    <row r="30" spans="2:3">
+      <c r="B30"/>
+    </row>
+    <row r="31" spans="2:3">
+      <c r="B31"/>
+    </row>
+    <row r="32" spans="2:3">
+      <c r="B32"/>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" s="22"/>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34"/>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35"/>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -2602,168 +2975,168 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19362CA-7547-47E7-8D6D-37E40A574CFD}">
   <dimension ref="B2:C29"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="2" max="2" width="9.3984375" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.09765625" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:3">
       <c r="B2" s="19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3">
+      <c r="B3" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="B4" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3">
+      <c r="B5" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3">
+      <c r="B6" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3">
+      <c r="B8" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3">
+      <c r="B9" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3">
+      <c r="B10" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3">
+      <c r="B11" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3">
+      <c r="B12" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3">
+      <c r="B14" s="19" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B3" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B4" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B5" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B6" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B7" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B8" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B9" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B10" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B11" s="9" t="s">
+    <row r="15" spans="2:3">
+      <c r="B15" s="19" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3">
+      <c r="B16" s="19" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" s="19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" s="19" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="19" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2">
+      <c r="B22" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="20" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B12" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B14" s="19" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B15" s="19" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B16" s="19" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B17" s="19" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B18" s="19" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B19" s="19" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B20" s="19" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B21" s="19" t="s">
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24" s="19" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B22" s="19" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B24" s="19" t="s">
+    <row r="25" spans="2:2">
+      <c r="B25" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B25" t="s">
+    <row r="26" spans="2:2">
+      <c r="B26" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B26" t="s">
+    <row r="27" spans="2:2">
+      <c r="B27" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B27" t="s">
+    <row r="28" spans="2:2">
+      <c r="B28" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B28" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:2">
       <c r="B29"/>
     </row>
   </sheetData>
@@ -2776,7 +3149,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{948DC7E8-6247-4DDA-A3B8-E05039F66E05}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2787,7 +3160,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33108BF5-BB5A-4329-8A3D-EFFA2011F4CC}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2798,7 +3171,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC2738DC-3A15-4BD1-8F4D-224529F6CE57}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>